<commit_message>
Swapped H1 and H2 spacebuses and rewired according to the swap.
Signed-off-by: Logan Tolbert <xem6df@virginia.edu>
</commit_message>
<xml_diff>
--- a/COMM_BOM.xlsx
+++ b/COMM_BOM.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\trebl\Desktop\UVA\MAE 4790\HEDGE2-COMM\COMM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3AFB681-3EE9-4664-B112-DB1B5AE293AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C560B74-3AB9-43AA-A34F-F024B25E0EA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="13200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-69" yWindow="-69" windowWidth="22080" windowHeight="13132" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="72">
   <si>
     <t>Id</t>
   </si>
@@ -233,6 +233,9 @@
   </si>
   <si>
     <t>https://www.mouser.com/ProductDetail/Coilcraft/XAL4040-103MEC?qs=zCSbvcPd3pYcdvH9kvmQzg%3D%3D</t>
+  </si>
+  <si>
+    <t>Footprint Size (Metric)</t>
   </si>
 </sst>
 </file>
@@ -283,9 +286,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyFill="1"/>
   </cellXfs>
@@ -591,14 +593,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:F25"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="2" max="2" width="37.4609375" customWidth="1"/>
-    <col min="4" max="4" width="39.921875" customWidth="1"/>
+    <col min="3" max="3" width="19.53515625" customWidth="1"/>
+    <col min="5" max="5" width="39.921875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -606,447 +609,486 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
+        <v>71</v>
+      </c>
+      <c r="D1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A2" s="1">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="1">
+      <c r="D2">
         <v>4</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>5</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A3" s="1">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A3">
         <v>16</v>
       </c>
       <c r="B3" t="s">
         <v>23</v>
       </c>
-      <c r="C3" s="1">
+      <c r="D3">
         <v>2</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>24</v>
       </c>
-      <c r="E3" t="s">
+      <c r="F3" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A4" s="1">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A4">
         <v>21</v>
       </c>
       <c r="B4" t="s">
         <v>31</v>
       </c>
-      <c r="C4" s="1">
-        <v>1</v>
-      </c>
-      <c r="D4" t="s">
+      <c r="C4">
+        <v>1608</v>
+      </c>
+      <c r="D4">
+        <v>1</v>
+      </c>
+      <c r="E4" t="s">
         <v>43</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="F4" s="1" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A5" s="1">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A5">
         <v>2</v>
       </c>
       <c r="B5" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="1">
+      <c r="C5">
+        <v>3216</v>
+      </c>
+      <c r="D5">
         <v>2</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
         <v>37</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="F5" s="1" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A6" s="1">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A6">
         <v>25</v>
       </c>
       <c r="B6" t="s">
         <v>36</v>
       </c>
-      <c r="C6" s="1">
-        <v>1</v>
-      </c>
-      <c r="D6" t="s">
+      <c r="C6">
+        <v>2012</v>
+      </c>
+      <c r="D6">
+        <v>1</v>
+      </c>
+      <c r="E6" t="s">
         <v>45</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="F6" s="1" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A7" s="1">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A7">
         <v>23</v>
       </c>
       <c r="B7" t="s">
         <v>33</v>
       </c>
-      <c r="C7" s="1">
-        <v>1</v>
-      </c>
-      <c r="D7" t="s">
+      <c r="C7">
+        <v>1005</v>
+      </c>
+      <c r="D7">
+        <v>1</v>
+      </c>
+      <c r="E7" t="s">
         <v>44</v>
       </c>
-      <c r="E7" s="2" t="s">
+      <c r="F7" s="1" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A8" s="1">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A8">
         <v>12</v>
       </c>
       <c r="B8" t="s">
         <v>19</v>
       </c>
-      <c r="C8" s="1">
-        <v>1</v>
-      </c>
-      <c r="D8" t="s">
+      <c r="C8">
+        <v>1608</v>
+      </c>
+      <c r="D8">
+        <v>1</v>
+      </c>
+      <c r="E8" t="s">
         <v>42</v>
       </c>
-      <c r="E8" s="2" t="s">
+      <c r="F8" s="1" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A9" s="1">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A9">
         <v>17</v>
       </c>
       <c r="B9" t="s">
         <v>10</v>
       </c>
-      <c r="C9" s="1">
-        <v>1</v>
-      </c>
-      <c r="D9" t="s">
+      <c r="C9">
+        <v>1005</v>
+      </c>
+      <c r="D9">
+        <v>1</v>
+      </c>
+      <c r="E9" t="s">
         <v>25</v>
       </c>
-      <c r="E9" s="2" t="s">
+      <c r="F9" s="1" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A10" s="1">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A10">
         <v>19</v>
       </c>
       <c r="B10" t="s">
         <v>10</v>
       </c>
-      <c r="C10" s="1">
-        <v>1</v>
-      </c>
-      <c r="D10" t="s">
+      <c r="C10">
+        <v>1005</v>
+      </c>
+      <c r="D10">
+        <v>1</v>
+      </c>
+      <c r="E10" t="s">
         <v>28</v>
       </c>
-      <c r="E10" s="2" t="s">
+      <c r="F10" s="1" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A11" s="1">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A11">
         <v>24</v>
       </c>
       <c r="B11" t="s">
         <v>34</v>
       </c>
-      <c r="C11" s="1">
-        <v>1</v>
-      </c>
-      <c r="D11" t="s">
+      <c r="C11">
+        <v>1608</v>
+      </c>
+      <c r="D11">
+        <v>1</v>
+      </c>
+      <c r="E11" t="s">
         <v>35</v>
       </c>
-      <c r="E11" s="2" t="s">
+      <c r="F11" s="1" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A12" s="1">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A12">
         <v>5</v>
       </c>
       <c r="B12" t="s">
         <v>10</v>
       </c>
-      <c r="C12" s="1">
+      <c r="C12">
+        <v>1005</v>
+      </c>
+      <c r="D12">
         <v>5</v>
       </c>
-      <c r="D12" t="s">
+      <c r="E12" t="s">
         <v>39</v>
       </c>
-      <c r="E12" s="2" t="s">
+      <c r="F12" s="1" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A13" s="1">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A13">
         <v>8</v>
       </c>
       <c r="B13" t="s">
         <v>13</v>
       </c>
-      <c r="C13" s="1">
+      <c r="C13">
+        <v>1005</v>
+      </c>
+      <c r="D13">
         <v>7</v>
       </c>
-      <c r="D13" t="s">
+      <c r="E13" t="s">
         <v>40</v>
       </c>
-      <c r="E13" s="2" t="s">
+      <c r="F13" s="1" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A14" s="1">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A14">
         <v>3</v>
       </c>
       <c r="B14" t="s">
         <v>7</v>
       </c>
-      <c r="C14" s="1">
-        <v>1</v>
-      </c>
-      <c r="D14" t="s">
+      <c r="C14">
+        <v>2012</v>
+      </c>
+      <c r="D14">
+        <v>1</v>
+      </c>
+      <c r="E14" t="s">
         <v>38</v>
       </c>
-      <c r="E14" s="2" t="s">
+      <c r="F14" s="1" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A15" s="1">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A15">
         <v>10</v>
       </c>
       <c r="B15" t="s">
         <v>16</v>
       </c>
-      <c r="C15" s="1">
-        <v>1</v>
-      </c>
-      <c r="D15" t="s">
+      <c r="C15">
+        <v>4040</v>
+      </c>
+      <c r="D15">
+        <v>1</v>
+      </c>
+      <c r="E15" t="s">
         <v>41</v>
       </c>
-      <c r="E15" s="2" t="s">
+      <c r="F15" s="1" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A16" s="1">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A16">
         <v>18</v>
       </c>
       <c r="B16" t="s">
         <v>26</v>
       </c>
-      <c r="C16" s="1">
-        <v>1</v>
-      </c>
-      <c r="D16" t="s">
+      <c r="D16">
+        <v>1</v>
+      </c>
+      <c r="E16" t="s">
         <v>27</v>
       </c>
-      <c r="E16" s="2" t="s">
+      <c r="F16" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A17" s="1">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A17">
         <v>4</v>
       </c>
       <c r="B17" t="s">
         <v>8</v>
       </c>
-      <c r="C17" s="1">
-        <v>1</v>
-      </c>
-      <c r="D17" t="s">
+      <c r="D17">
+        <v>1</v>
+      </c>
+      <c r="E17" t="s">
         <v>9</v>
       </c>
-      <c r="E17" s="2" t="s">
+      <c r="F17" s="1" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A18" s="1">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A18">
         <v>6</v>
       </c>
       <c r="B18" t="s">
         <v>8</v>
       </c>
-      <c r="C18" s="1">
+      <c r="D18">
         <v>2</v>
       </c>
-      <c r="D18" t="s">
+      <c r="E18" t="s">
         <v>54</v>
       </c>
-      <c r="E18" s="2" t="s">
+      <c r="F18" s="1" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A19" s="1">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A19">
         <v>15</v>
       </c>
       <c r="B19" t="s">
         <v>8</v>
       </c>
-      <c r="C19" s="1">
-        <v>1</v>
-      </c>
-      <c r="D19" t="s">
+      <c r="D19">
+        <v>1</v>
+      </c>
+      <c r="E19" t="s">
         <v>22</v>
       </c>
-      <c r="E19" s="2" t="s">
+      <c r="F19" s="1" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A20" s="1">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A20">
         <v>22</v>
       </c>
       <c r="B20" t="s">
         <v>32</v>
       </c>
-      <c r="C20" s="1">
-        <v>1</v>
-      </c>
-      <c r="D20" t="s">
+      <c r="D20">
+        <v>1</v>
+      </c>
+      <c r="E20" t="s">
         <v>32</v>
       </c>
-      <c r="E20" s="2" t="s">
+      <c r="F20" s="1" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A21" s="1">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A21">
         <v>7</v>
       </c>
       <c r="B21" t="s">
         <v>11</v>
       </c>
-      <c r="C21" s="1">
-        <v>1</v>
-      </c>
-      <c r="D21" t="s">
+      <c r="D21">
+        <v>1</v>
+      </c>
+      <c r="E21" t="s">
         <v>12</v>
       </c>
-      <c r="E21" s="3" t="s">
+      <c r="F21" s="2" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A22" s="1">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A22">
         <v>20</v>
       </c>
       <c r="B22" t="s">
         <v>29</v>
       </c>
-      <c r="C22" s="1">
-        <v>1</v>
-      </c>
-      <c r="D22" t="s">
+      <c r="D22">
+        <v>1</v>
+      </c>
+      <c r="E22" t="s">
         <v>30</v>
       </c>
-      <c r="E22" s="2" t="s">
+      <c r="F22" s="1" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A23" s="1">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A23">
         <v>11</v>
       </c>
       <c r="B23" t="s">
         <v>17</v>
       </c>
-      <c r="C23" s="1">
-        <v>1</v>
-      </c>
-      <c r="D23" t="s">
+      <c r="D23">
+        <v>1</v>
+      </c>
+      <c r="E23" t="s">
         <v>18</v>
       </c>
-      <c r="E23" s="2" t="s">
+      <c r="F23" s="1" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A24" s="1">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A24">
         <v>9</v>
       </c>
       <c r="B24" t="s">
         <v>14</v>
       </c>
-      <c r="C24" s="1">
-        <v>1</v>
-      </c>
-      <c r="D24" t="s">
+      <c r="D24">
+        <v>1</v>
+      </c>
+      <c r="E24" t="s">
         <v>15</v>
       </c>
-      <c r="E24" s="2" t="s">
+      <c r="F24" s="1" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A25" s="1">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A25">
         <v>13</v>
       </c>
       <c r="B25" t="s">
         <v>20</v>
       </c>
-      <c r="C25" s="1">
-        <v>1</v>
-      </c>
-      <c r="D25" t="s">
+      <c r="D25">
+        <v>1</v>
+      </c>
+      <c r="E25" t="s">
         <v>21</v>
       </c>
-      <c r="E25" s="2" t="s">
+      <c r="F25" s="1" t="s">
         <v>63</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="E16" r:id="rId1" xr:uid="{326213F1-EA96-4940-B57C-6B62601104FE}"/>
-    <hyperlink ref="E5" r:id="rId2" xr:uid="{8CE27A86-DD92-4B1E-BF53-77BEFD627EA2}"/>
-    <hyperlink ref="E4" r:id="rId3" xr:uid="{53EC14E4-DD55-4C48-BB9D-6351A9B0B30C}"/>
-    <hyperlink ref="E6" r:id="rId4" xr:uid="{F614837E-C79B-4D04-9507-3FF1FBC2FCA0}"/>
-    <hyperlink ref="E19" r:id="rId5" xr:uid="{2CED2099-8068-4901-994B-895A5B80DA4B}"/>
-    <hyperlink ref="E17" r:id="rId6" xr:uid="{7169CF27-8DD4-47B4-BF5F-6AEEAD48D0D9}"/>
-    <hyperlink ref="E18" r:id="rId7" xr:uid="{9D82EC78-5106-4641-B34F-D0A3E2C02F5A}"/>
-    <hyperlink ref="E7" r:id="rId8" xr:uid="{7BE9A0CB-8212-472F-9843-565DC92235F3}"/>
-    <hyperlink ref="E8" r:id="rId9" xr:uid="{9D9300C3-BBA2-44FC-AA50-AEE94EE72B5C}"/>
-    <hyperlink ref="E21" r:id="rId10" xr:uid="{71DCB31B-DAA7-49BA-B966-158BE3FA19E9}"/>
-    <hyperlink ref="E20" r:id="rId11" xr:uid="{41F70F48-F6CA-41CD-9151-109073AA2FF2}"/>
-    <hyperlink ref="E22" r:id="rId12" xr:uid="{1F9438C1-60AC-4D30-B005-BEB534CCFD79}"/>
-    <hyperlink ref="E23" r:id="rId13" xr:uid="{4D1495E3-3E65-4249-8F9B-AA1913F9831F}"/>
-    <hyperlink ref="E24" r:id="rId14" xr:uid="{976FDE44-A317-4092-B5B1-1F1673DE1E8D}"/>
-    <hyperlink ref="E25" r:id="rId15" xr:uid="{ADCB232E-4B69-40D6-85D3-F81A00C5FF21}"/>
-    <hyperlink ref="E14" r:id="rId16" xr:uid="{7F9FDE33-9516-4F13-BBFA-BE5BC54A2288}"/>
-    <hyperlink ref="E11" r:id="rId17" xr:uid="{1E8B52FF-7CC8-4B1D-9FA6-991D93FE6FD0}"/>
-    <hyperlink ref="E10" r:id="rId18" xr:uid="{0B1335B6-B4D1-44AC-98B7-F8ACDD550290}"/>
-    <hyperlink ref="E9" r:id="rId19" xr:uid="{2E3081D2-D803-40D5-BEA7-6B5B8B92A8C7}"/>
-    <hyperlink ref="E12" r:id="rId20" xr:uid="{02CFAEB8-58D3-4517-87AF-1E91E55FB1E1}"/>
-    <hyperlink ref="E13" r:id="rId21" xr:uid="{8C2D8ABC-9CAD-48DD-BCBC-7B3AD60D46AE}"/>
-    <hyperlink ref="E15" r:id="rId22" xr:uid="{376FA2EB-B6A8-4E58-8140-60C154FD6815}"/>
+    <hyperlink ref="F16" r:id="rId1" xr:uid="{326213F1-EA96-4940-B57C-6B62601104FE}"/>
+    <hyperlink ref="F5" r:id="rId2" xr:uid="{8CE27A86-DD92-4B1E-BF53-77BEFD627EA2}"/>
+    <hyperlink ref="F4" r:id="rId3" xr:uid="{53EC14E4-DD55-4C48-BB9D-6351A9B0B30C}"/>
+    <hyperlink ref="F6" r:id="rId4" xr:uid="{F614837E-C79B-4D04-9507-3FF1FBC2FCA0}"/>
+    <hyperlink ref="F19" r:id="rId5" xr:uid="{2CED2099-8068-4901-994B-895A5B80DA4B}"/>
+    <hyperlink ref="F17" r:id="rId6" xr:uid="{7169CF27-8DD4-47B4-BF5F-6AEEAD48D0D9}"/>
+    <hyperlink ref="F18" r:id="rId7" xr:uid="{9D82EC78-5106-4641-B34F-D0A3E2C02F5A}"/>
+    <hyperlink ref="F7" r:id="rId8" xr:uid="{7BE9A0CB-8212-472F-9843-565DC92235F3}"/>
+    <hyperlink ref="F8" r:id="rId9" xr:uid="{9D9300C3-BBA2-44FC-AA50-AEE94EE72B5C}"/>
+    <hyperlink ref="F21" r:id="rId10" xr:uid="{71DCB31B-DAA7-49BA-B966-158BE3FA19E9}"/>
+    <hyperlink ref="F20" r:id="rId11" xr:uid="{41F70F48-F6CA-41CD-9151-109073AA2FF2}"/>
+    <hyperlink ref="F22" r:id="rId12" xr:uid="{1F9438C1-60AC-4D30-B005-BEB534CCFD79}"/>
+    <hyperlink ref="F23" r:id="rId13" xr:uid="{4D1495E3-3E65-4249-8F9B-AA1913F9831F}"/>
+    <hyperlink ref="F24" r:id="rId14" xr:uid="{976FDE44-A317-4092-B5B1-1F1673DE1E8D}"/>
+    <hyperlink ref="F25" r:id="rId15" xr:uid="{ADCB232E-4B69-40D6-85D3-F81A00C5FF21}"/>
+    <hyperlink ref="F14" r:id="rId16" xr:uid="{7F9FDE33-9516-4F13-BBFA-BE5BC54A2288}"/>
+    <hyperlink ref="F11" r:id="rId17" xr:uid="{1E8B52FF-7CC8-4B1D-9FA6-991D93FE6FD0}"/>
+    <hyperlink ref="F10" r:id="rId18" xr:uid="{0B1335B6-B4D1-44AC-98B7-F8ACDD550290}"/>
+    <hyperlink ref="F9" r:id="rId19" xr:uid="{2E3081D2-D803-40D5-BEA7-6B5B8B92A8C7}"/>
+    <hyperlink ref="F12" r:id="rId20" xr:uid="{02CFAEB8-58D3-4517-87AF-1E91E55FB1E1}"/>
+    <hyperlink ref="F13" r:id="rId21" xr:uid="{8C2D8ABC-9CAD-48DD-BCBC-7B3AD60D46AE}"/>
+    <hyperlink ref="F15" r:id="rId22" xr:uid="{376FA2EB-B6A8-4E58-8140-60C154FD6815}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>